<commit_message>
Add Tr4 Mutant Vehicle SOI SOP and update ToC
Documents the annual BMorg MVSOI submission process for SirKiss.
Includes 2026 reference answers, timeline, submission steps, and
contacts. ToC updated with Tr4 entry.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Standard Operating Procedures/SOPs Table of Contents.xlsx
+++ b/Standard Operating Procedures/SOPs Table of Contents.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="14.75" customWidth="1" style="16" min="2" max="2"/>
@@ -665,42 +665,45 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n"/>
-      <c r="E13" s="11" t="n"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Tr4</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Mutant Vehicle Statement of Intent (BMorg)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="12" t="n"/>
+      <c r="E14" s="11" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Art Car</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>SirKiss Setup and Operation, parts list</t>
-        </is>
-      </c>
-      <c r="E14" s="11" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>AC2</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>Sound System</t>
         </is>
       </c>
       <c r="E15" s="11" t="n"/>
@@ -709,45 +712,45 @@
       <c r="A16" s="12" t="n"/>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC2</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>Generator Spec Sheet, parts list, PM checklist</t>
+          <t>Sound System</t>
         </is>
       </c>
       <c r="E16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="12" t="n"/>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Facilities</t>
-        </is>
-      </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Fc1</t>
+          <t>AC3</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>Plumbing Diagram, parts list</t>
+          <t>Generator Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="12" t="n"/>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Facilities</t>
+        </is>
+      </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Fc2</t>
+          <t>Fc1</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Supplies Shopping List</t>
+          <t>Plumbing Diagram, parts list</t>
         </is>
       </c>
       <c r="E18" s="11" t="n"/>
@@ -756,40 +759,40 @@
       <c r="A19" s="12" t="n"/>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Fc3</t>
+          <t>Fc2</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>Supplies Shopping List</t>
         </is>
       </c>
       <c r="E19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="n"/>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>Maintenance</t>
-        </is>
-      </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>PM1</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>Isuzu Spec Sheet, parts list, PM checklist</t>
+          <t>Fc3</t>
         </is>
       </c>
       <c r="E20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="12" t="n"/>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>PM2</t>
+          <t>PM1</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>Refrigeration Trailer Spec Sheet, parts list, PM checklist</t>
+          <t>Isuzu Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E21" s="11" t="n"/>
@@ -798,12 +801,12 @@
       <c r="A22" s="12" t="n"/>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>PM3</t>
+          <t>PM2</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Cargo Trailer Spec Sheet, parts list, PM checklist</t>
+          <t>Refrigeration Trailer Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E22" s="11" t="n"/>
@@ -812,12 +815,12 @@
       <c r="A23" s="12" t="n"/>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>PM4</t>
+          <t>PM3</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>Porta Potties Trailer Spec Sheet, parts list, PM checklist</t>
+          <t>Cargo Trailer Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E23" s="11" t="n"/>
@@ -826,45 +829,45 @@
       <c r="A24" s="12" t="n"/>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>PM5</t>
+          <t>PM4</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>Generator Trailer Spec Sheet, parts list, PM checklist</t>
+          <t>Porta Potties Trailer Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="12" t="n"/>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>Power Grid</t>
-        </is>
-      </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Pow1</t>
+          <t>PM5</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>Grid Scamatics</t>
+          <t>Generator Trailer Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="12" t="n"/>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Power Grid</t>
+        </is>
+      </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Pow2</t>
+          <t>Pow1</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>Generator Spec Sheet, parts list, PM checklist</t>
+          <t>Grid Scamatics</t>
         </is>
       </c>
       <c r="E26" s="11" t="n"/>
@@ -873,45 +876,45 @@
       <c r="A27" s="12" t="n"/>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Pow3</t>
+          <t>Pow2</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>Fuel Containment</t>
+          <t>Generator Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="12" t="n"/>
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>Shelter</t>
-        </is>
-      </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Sh1</t>
+          <t>Pow3</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>Shade Structure Setup, parts list</t>
+          <t>Fuel Containment</t>
         </is>
       </c>
       <c r="E28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="12" t="n"/>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Shelter</t>
+        </is>
+      </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Sh2</t>
+          <t>Sh1</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>Sound System</t>
+          <t>Shade Structure Setup, parts list</t>
         </is>
       </c>
       <c r="E29" s="11" t="n"/>
@@ -920,18 +923,28 @@
       <c r="A30" s="12" t="n"/>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Sh3</t>
+          <t>Sh2</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Fire Poofer</t>
+          <t>Sound System</t>
         </is>
       </c>
       <c r="E30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="12" t="n"/>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Sh3</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>Fire Poofer</t>
+        </is>
+      </c>
       <c r="E31" s="11" t="n"/>
     </row>
     <row r="32">
@@ -939,57 +952,42 @@
       <c r="E32" s="11" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="12" t="inlineStr">
+      <c r="A33" s="12" t="n"/>
+      <c r="E33" s="11" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t>Committees</t>
         </is>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>Logistics</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>Log1</t>
         </is>
       </c>
-      <c r="D33" s="10" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
         <is>
           <t>Trailer Hitch &amp; GVW Specs</t>
-        </is>
-      </c>
-      <c r="E33" s="11" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="12" t="n"/>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>Log2</t>
-        </is>
-      </c>
-      <c r="D34" s="10" t="inlineStr">
-        <is>
-          <t>Camp Layout Map</t>
         </is>
       </c>
       <c r="E34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="12" t="n"/>
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>Safe1</t>
+          <t>Log2</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>Hazards and Training</t>
+          <t>Camp Layout Map</t>
         </is>
       </c>
       <c r="E35" s="11" t="n"/>
@@ -998,31 +996,36 @@
       <c r="A36" s="12" t="n"/>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Kch1</t>
+          <t>Safe1</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>Kitchen Layout</t>
+          <t>Hazards and Training</t>
         </is>
       </c>
       <c r="E36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="12" t="n"/>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>Kch2</t>
+          <t>Kch1</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>Health Department Compliance</t>
+          <t>Kitchen Layout</t>
         </is>
       </c>
       <c r="E37" s="11" t="n"/>
@@ -1031,45 +1034,45 @@
       <c r="A38" s="12" t="n"/>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>Kch3</t>
+          <t>Kch2</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>Food Menu and Shopping List</t>
+          <t>Health Department Compliance</t>
         </is>
       </c>
       <c r="E38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="12" t="n"/>
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t>Bar &amp; Beverage</t>
-        </is>
-      </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>Bev1</t>
+          <t>Kch3</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>Keg Trailer Systems</t>
+          <t>Food Menu and Shopping List</t>
         </is>
       </c>
       <c r="E39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="12" t="n"/>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Bar &amp; Beverage</t>
+        </is>
+      </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>Bev2</t>
+          <t>Bev1</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>Keg Filling</t>
+          <t>Keg Trailer Systems</t>
         </is>
       </c>
       <c r="E40" s="11" t="n"/>
@@ -1078,31 +1081,26 @@
       <c r="A41" s="12" t="n"/>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>Bev3</t>
+          <t>Bev2</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>Beverage Menu and Shopping List</t>
+          <t>Keg Filling</t>
         </is>
       </c>
       <c r="E41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="12" t="n"/>
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>Events</t>
-        </is>
-      </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>Eve1</t>
+          <t>Bev3</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>Signup Monkey</t>
+          <t>Beverage Menu and Shopping List</t>
         </is>
       </c>
       <c r="E42" s="11" t="n"/>
@@ -1111,12 +1109,12 @@
       <c r="A43" s="12" t="n"/>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>Events</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>LNT1</t>
+          <t>Eve1</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
@@ -1128,6 +1126,21 @@
     </row>
     <row r="44">
       <c r="A44" s="12" t="n"/>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>LNT</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>LNT1</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>Signup Monkey</t>
+        </is>
+      </c>
       <c r="E44" s="11" t="n"/>
     </row>
     <row r="45">
@@ -1163,11 +1176,15 @@
       <c r="E52" s="11" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="13" t="n"/>
-      <c r="B53" s="14" t="n"/>
-      <c r="C53" s="14" t="n"/>
-      <c r="D53" s="14" t="n"/>
-      <c r="E53" s="15" t="n"/>
+      <c r="A53" s="12" t="n"/>
+      <c r="E53" s="11" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="13" t="n"/>
+      <c r="B54" s="14" t="n"/>
+      <c r="C54" s="14" t="n"/>
+      <c r="D54" s="14" t="n"/>
+      <c r="E54" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Add Com1 Slack, Com2 Sakari, Com3 HubSpot SOPs; update ToC
Split the Communications Officer SOP pack into three individual SOPs.
Com1 covers Slack structure, posting rules, and meeting recap template.
Com2 covers Sakari SMS campaigns and 1:1 texting.
Com3 covers HubSpot CRM, forms, lists, email, website, and handoff.
ToC updated with dates for all three.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Standard Operating Procedures/SOPs Table of Contents.xlsx
+++ b/Standard Operating Procedures/SOPs Table of Contents.xlsx
@@ -541,7 +541,11 @@
           <t>Slack</t>
         </is>
       </c>
-      <c r="E4" s="11" t="n"/>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="n"/>
@@ -555,7 +559,11 @@
           <t>Sakari</t>
         </is>
       </c>
-      <c r="E5" s="11" t="n"/>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="n"/>
@@ -569,7 +577,11 @@
           <t>HubSpot</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n"/>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="n"/>
@@ -665,17 +677,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>Tr4</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>Mutant Vehicle Statement of Intent (BMorg)</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>

</xml_diff>

<commit_message>
Add Tr2 IRS 509(a)(2) Administration SOP; update ToC
Documents EIN 99-1556119, 501(c)(3)/509(a)(2) status, Form 990 filing
deadlines (June 15, FYE Jan 31), annual compliance checklist, 7-year
record retention, and IRS contact info from the 2024 determination letter.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Standard Operating Procedures/SOPs Table of Contents.xlsx
+++ b/Standard Operating Procedures/SOPs Table of Contents.xlsx
@@ -653,10 +653,14 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>501c3 Administration</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="n"/>
+          <t>IRS 509(a)(2) Administration</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="n"/>

</xml_diff>

<commit_message>
Add Com4 Role Email Address Setup SOP
New SOP covering end-to-end process for creating role-based email addresses: Cloudflare routing rule, Gmail forwarding verification, label/filter setup, and Send As configuration. TOC updated with Com4 entry.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Standard Operating Procedures/SOPs Table of Contents.xlsx
+++ b/Standard Operating Procedures/SOPs Table of Contents.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="14.75" customWidth="1" style="16" min="2" max="2"/>
@@ -584,34 +584,37 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n"/>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Human Resources</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>HR1</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>Onboarding Questionaire</t>
-        </is>
-      </c>
-      <c r="E7" s="11" t="n"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Com4</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Role Email Address Setup</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="n"/>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Human Resources</t>
+        </is>
+      </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>HR2</t>
+          <t>HR1</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Camp Integration and FAQs</t>
+          <t>Onboarding Questionaire</t>
         </is>
       </c>
       <c r="E8" s="11" t="n"/>
@@ -620,120 +623,120 @@
       <c r="A9" s="12" t="n"/>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>HR3</t>
+          <t>HR2</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Camp Integration and FAQs</t>
         </is>
       </c>
       <c r="E9" s="11" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="n"/>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Treasurer</t>
-        </is>
-      </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Tr1</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>Accounting and Budgets</t>
+          <t>HR3</t>
         </is>
       </c>
       <c r="E10" s="11" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="12" t="n"/>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Treasurer</t>
+        </is>
+      </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Tr2</t>
+          <t>Tr1</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>IRS 509(a)(2) Administration</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>2026-03-04</t>
-        </is>
-      </c>
+          <t>Accounting and Budgets</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="n"/>
       <c r="C12" s="10" t="inlineStr">
         <is>
+          <t>Tr2</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>IRS 509(a)(2) Administration</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n"/>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
           <t>Tr3</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>Statement of Intent (BMorg)</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="C13" s="0" t="inlineStr">
+    <row r="14">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>Tr4</t>
         </is>
       </c>
-      <c r="D13" s="0" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>Mutant Vehicle Statement of Intent (BMorg)</t>
         </is>
       </c>
-      <c r="E13" s="0" t="inlineStr">
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="12" t="n"/>
-      <c r="E14" s="11" t="n"/>
-    </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="12" t="n"/>
+      <c r="E15" s="11" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Art Car</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>SirKiss Setup and Operation, parts list</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>AC2</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>Sound System</t>
         </is>
       </c>
       <c r="E16" s="11" t="n"/>
@@ -742,45 +745,45 @@
       <c r="A17" s="12" t="n"/>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC2</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>Generator Spec Sheet, parts list, PM checklist</t>
+          <t>Sound System</t>
         </is>
       </c>
       <c r="E17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="12" t="n"/>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Facilities</t>
-        </is>
-      </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Fc1</t>
+          <t>AC3</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Plumbing Diagram, parts list</t>
+          <t>Generator Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="12" t="n"/>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Facilities</t>
+        </is>
+      </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Fc2</t>
+          <t>Fc1</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>Supplies Shopping List</t>
+          <t>Plumbing Diagram, parts list</t>
         </is>
       </c>
       <c r="E19" s="11" t="n"/>
@@ -789,40 +792,40 @@
       <c r="A20" s="12" t="n"/>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Fc3</t>
+          <t>Fc2</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Supplies Shopping List</t>
         </is>
       </c>
       <c r="E20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="12" t="n"/>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>Maintenance</t>
-        </is>
-      </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>PM1</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>Isuzu Spec Sheet, parts list, PM checklist</t>
+          <t>Fc3</t>
         </is>
       </c>
       <c r="E21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="12" t="n"/>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>PM2</t>
+          <t>PM1</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Refrigeration Trailer Spec Sheet, parts list, PM checklist</t>
+          <t>Isuzu Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E22" s="11" t="n"/>
@@ -831,12 +834,12 @@
       <c r="A23" s="12" t="n"/>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>PM3</t>
+          <t>PM2</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>Cargo Trailer Spec Sheet, parts list, PM checklist</t>
+          <t>Refrigeration Trailer Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E23" s="11" t="n"/>
@@ -845,12 +848,12 @@
       <c r="A24" s="12" t="n"/>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>PM4</t>
+          <t>PM3</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>Porta Potties Trailer Spec Sheet, parts list, PM checklist</t>
+          <t>Cargo Trailer Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E24" s="11" t="n"/>
@@ -859,45 +862,45 @@
       <c r="A25" s="12" t="n"/>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>PM5</t>
+          <t>PM4</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>Generator Trailer Spec Sheet, parts list, PM checklist</t>
+          <t>Porta Potties Trailer Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="12" t="n"/>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>Power Grid</t>
-        </is>
-      </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Pow1</t>
+          <t>PM5</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>Grid Scamatics</t>
+          <t>Generator Trailer Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="12" t="n"/>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Power Grid</t>
+        </is>
+      </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Pow2</t>
+          <t>Pow1</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>Generator Spec Sheet, parts list, PM checklist</t>
+          <t>Grid Scamatics</t>
         </is>
       </c>
       <c r="E27" s="11" t="n"/>
@@ -906,45 +909,45 @@
       <c r="A28" s="12" t="n"/>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Pow3</t>
+          <t>Pow2</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>Fuel Containment</t>
+          <t>Generator Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="12" t="n"/>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Shelter</t>
-        </is>
-      </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Sh1</t>
+          <t>Pow3</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>Shade Structure Setup, parts list</t>
+          <t>Fuel Containment</t>
         </is>
       </c>
       <c r="E29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="12" t="n"/>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Shelter</t>
+        </is>
+      </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Sh2</t>
+          <t>Sh1</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Sound System</t>
+          <t>Shade Structure Setup, parts list</t>
         </is>
       </c>
       <c r="E30" s="11" t="n"/>
@@ -953,18 +956,28 @@
       <c r="A31" s="12" t="n"/>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>Sh3</t>
+          <t>Sh2</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Fire Poofer</t>
+          <t>Sound System</t>
         </is>
       </c>
       <c r="E31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="12" t="n"/>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Sh3</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Fire Poofer</t>
+        </is>
+      </c>
       <c r="E32" s="11" t="n"/>
     </row>
     <row r="33">
@@ -972,57 +985,42 @@
       <c r="E33" s="11" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="inlineStr">
+      <c r="A34" s="12" t="n"/>
+      <c r="E34" s="11" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>Committees</t>
         </is>
       </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>Logistics</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr">
+      <c r="C35" s="10" t="inlineStr">
         <is>
           <t>Log1</t>
         </is>
       </c>
-      <c r="D34" s="10" t="inlineStr">
+      <c r="D35" s="10" t="inlineStr">
         <is>
           <t>Trailer Hitch &amp; GVW Specs</t>
-        </is>
-      </c>
-      <c r="E34" s="11" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="12" t="n"/>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>Log2</t>
-        </is>
-      </c>
-      <c r="D35" s="10" t="inlineStr">
-        <is>
-          <t>Camp Layout Map</t>
         </is>
       </c>
       <c r="E35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="12" t="n"/>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Safe1</t>
+          <t>Log2</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>Hazards and Training</t>
+          <t>Camp Layout Map</t>
         </is>
       </c>
       <c r="E36" s="11" t="n"/>
@@ -1031,31 +1029,36 @@
       <c r="A37" s="12" t="n"/>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>Kch1</t>
+          <t>Safe1</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>Kitchen Layout</t>
+          <t>Hazards and Training</t>
         </is>
       </c>
       <c r="E37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="12" t="n"/>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>Kch2</t>
+          <t>Kch1</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>Health Department Compliance</t>
+          <t>Kitchen Layout</t>
         </is>
       </c>
       <c r="E38" s="11" t="n"/>
@@ -1064,45 +1067,45 @@
       <c r="A39" s="12" t="n"/>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>Kch3</t>
+          <t>Kch2</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>Food Menu and Shopping List</t>
+          <t>Health Department Compliance</t>
         </is>
       </c>
       <c r="E39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="12" t="n"/>
-      <c r="B40" s="10" t="inlineStr">
-        <is>
-          <t>Bar &amp; Beverage</t>
-        </is>
-      </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>Bev1</t>
+          <t>Kch3</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>Keg Trailer Systems</t>
+          <t>Food Menu and Shopping List</t>
         </is>
       </c>
       <c r="E40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="12" t="n"/>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Bar &amp; Beverage</t>
+        </is>
+      </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>Bev2</t>
+          <t>Bev1</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>Keg Filling</t>
+          <t>Keg Trailer Systems</t>
         </is>
       </c>
       <c r="E41" s="11" t="n"/>
@@ -1111,31 +1114,26 @@
       <c r="A42" s="12" t="n"/>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>Bev3</t>
+          <t>Bev2</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>Beverage Menu and Shopping List</t>
+          <t>Keg Filling</t>
         </is>
       </c>
       <c r="E42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="12" t="n"/>
-      <c r="B43" s="10" t="inlineStr">
-        <is>
-          <t>Events</t>
-        </is>
-      </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>Eve1</t>
+          <t>Bev3</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>Signup Monkey</t>
+          <t>Beverage Menu and Shopping List</t>
         </is>
       </c>
       <c r="E43" s="11" t="n"/>
@@ -1144,12 +1142,12 @@
       <c r="A44" s="12" t="n"/>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>Events</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>LNT1</t>
+          <t>Eve1</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
@@ -1161,6 +1159,21 @@
     </row>
     <row r="45">
       <c r="A45" s="12" t="n"/>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>LNT</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>LNT1</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>Signup Monkey</t>
+        </is>
+      </c>
       <c r="E45" s="11" t="n"/>
     </row>
     <row r="46">
@@ -1196,11 +1209,15 @@
       <c r="E53" s="11" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="13" t="n"/>
-      <c r="B54" s="14" t="n"/>
-      <c r="C54" s="14" t="n"/>
-      <c r="D54" s="14" t="n"/>
-      <c r="E54" s="15" t="n"/>
+      <c r="A54" s="12" t="n"/>
+      <c r="E54" s="11" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="13" t="n"/>
+      <c r="B55" s="14" t="n"/>
+      <c r="C55" s="14" t="n"/>
+      <c r="D55" s="14" t="n"/>
+      <c r="E55" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Add Tr5 Hell Station Petrol Application SOP; update ToC
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Standard Operating Procedures/SOPs Table of Contents.xlsx
+++ b/Standard Operating Procedures/SOPs Table of Contents.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="14.75" customWidth="1" style="16" min="2" max="2"/>
@@ -584,17 +584,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>Com4</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>Role Email Address Setup</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="0" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
@@ -715,42 +715,45 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="E15" s="11" t="n"/>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>Tr5</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>Hell Station Petrol Application (BMorg)</t>
+        </is>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="12" t="n"/>
+      <c r="E16" s="11" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Infrastructure</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Art Car</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>SirKiss Setup and Operation, parts list</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="n"/>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>AC2</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>Sound System</t>
         </is>
       </c>
       <c r="E17" s="11" t="n"/>
@@ -759,45 +762,45 @@
       <c r="A18" s="12" t="n"/>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC2</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Generator Spec Sheet, parts list, PM checklist</t>
+          <t>Sound System</t>
         </is>
       </c>
       <c r="E18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="12" t="n"/>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>Facilities</t>
-        </is>
-      </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Fc1</t>
+          <t>AC3</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>Plumbing Diagram, parts list</t>
+          <t>Generator Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="n"/>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Facilities</t>
+        </is>
+      </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Fc2</t>
+          <t>Fc1</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>Supplies Shopping List</t>
+          <t>Plumbing Diagram, parts list</t>
         </is>
       </c>
       <c r="E20" s="11" t="n"/>
@@ -806,40 +809,40 @@
       <c r="A21" s="12" t="n"/>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Fc3</t>
+          <t>Fc2</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>Supplies Shopping List</t>
         </is>
       </c>
       <c r="E21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="12" t="n"/>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>Maintenance</t>
-        </is>
-      </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>PM1</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>Isuzu Spec Sheet, parts list, PM checklist</t>
+          <t>Fc3</t>
         </is>
       </c>
       <c r="E22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="12" t="n"/>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>PM2</t>
+          <t>PM1</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>Refrigeration Trailer Spec Sheet, parts list, PM checklist</t>
+          <t>Isuzu Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E23" s="11" t="n"/>
@@ -848,12 +851,12 @@
       <c r="A24" s="12" t="n"/>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>PM3</t>
+          <t>PM2</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>Cargo Trailer Spec Sheet, parts list, PM checklist</t>
+          <t>Refrigeration Trailer Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E24" s="11" t="n"/>
@@ -862,12 +865,12 @@
       <c r="A25" s="12" t="n"/>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>PM4</t>
+          <t>PM3</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>Porta Potties Trailer Spec Sheet, parts list, PM checklist</t>
+          <t>Cargo Trailer Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E25" s="11" t="n"/>
@@ -876,45 +879,45 @@
       <c r="A26" s="12" t="n"/>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>PM5</t>
+          <t>PM4</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>Generator Trailer Spec Sheet, parts list, PM checklist</t>
+          <t>Porta Potties Trailer Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="12" t="n"/>
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t>Power Grid</t>
-        </is>
-      </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Pow1</t>
+          <t>PM5</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>Grid Scamatics</t>
+          <t>Generator Trailer Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="12" t="n"/>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Power Grid</t>
+        </is>
+      </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Pow2</t>
+          <t>Pow1</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>Generator Spec Sheet, parts list, PM checklist</t>
+          <t>Grid Scamatics</t>
         </is>
       </c>
       <c r="E28" s="11" t="n"/>
@@ -923,45 +926,45 @@
       <c r="A29" s="12" t="n"/>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Pow3</t>
+          <t>Pow2</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>Fuel Containment</t>
+          <t>Generator Spec Sheet, parts list, PM checklist</t>
         </is>
       </c>
       <c r="E29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="12" t="n"/>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>Shelter</t>
-        </is>
-      </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Sh1</t>
+          <t>Pow3</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Shade Structure Setup, parts list</t>
+          <t>Fuel Containment</t>
         </is>
       </c>
       <c r="E30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="12" t="n"/>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Shelter</t>
+        </is>
+      </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>Sh2</t>
+          <t>Sh1</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Sound System</t>
+          <t>Shade Structure Setup, parts list</t>
         </is>
       </c>
       <c r="E31" s="11" t="n"/>
@@ -970,18 +973,28 @@
       <c r="A32" s="12" t="n"/>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Sh3</t>
+          <t>Sh2</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>Fire Poofer</t>
+          <t>Sound System</t>
         </is>
       </c>
       <c r="E32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="12" t="n"/>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Sh3</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Fire Poofer</t>
+        </is>
+      </c>
       <c r="E33" s="11" t="n"/>
     </row>
     <row r="34">
@@ -989,57 +1002,42 @@
       <c r="E34" s="11" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="12" t="inlineStr">
+      <c r="A35" s="12" t="n"/>
+      <c r="E35" s="11" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t>Committees</t>
         </is>
       </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>Logistics</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>Log1</t>
         </is>
       </c>
-      <c r="D35" s="10" t="inlineStr">
+      <c r="D36" s="10" t="inlineStr">
         <is>
           <t>Trailer Hitch &amp; GVW Specs</t>
-        </is>
-      </c>
-      <c r="E35" s="11" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="12" t="n"/>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>Log2</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t>Camp Layout Map</t>
         </is>
       </c>
       <c r="E36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="12" t="n"/>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>Safe1</t>
+          <t>Log2</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>Hazards and Training</t>
+          <t>Camp Layout Map</t>
         </is>
       </c>
       <c r="E37" s="11" t="n"/>
@@ -1048,31 +1046,36 @@
       <c r="A38" s="12" t="n"/>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Kitchen</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>Kch1</t>
+          <t>Safe1</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>Kitchen Layout</t>
+          <t>Hazards and Training</t>
         </is>
       </c>
       <c r="E38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="12" t="n"/>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen</t>
+        </is>
+      </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>Kch2</t>
+          <t>Kch1</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>Health Department Compliance</t>
+          <t>Kitchen Layout</t>
         </is>
       </c>
       <c r="E39" s="11" t="n"/>
@@ -1081,45 +1084,45 @@
       <c r="A40" s="12" t="n"/>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>Kch3</t>
+          <t>Kch2</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>Food Menu and Shopping List</t>
+          <t>Health Department Compliance</t>
         </is>
       </c>
       <c r="E40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="12" t="n"/>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>Bar &amp; Beverage</t>
-        </is>
-      </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>Bev1</t>
+          <t>Kch3</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>Keg Trailer Systems</t>
+          <t>Food Menu and Shopping List</t>
         </is>
       </c>
       <c r="E41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="12" t="n"/>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>Bar &amp; Beverage</t>
+        </is>
+      </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>Bev2</t>
+          <t>Bev1</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>Keg Filling</t>
+          <t>Keg Trailer Systems</t>
         </is>
       </c>
       <c r="E42" s="11" t="n"/>
@@ -1128,31 +1131,26 @@
       <c r="A43" s="12" t="n"/>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>Bev3</t>
+          <t>Bev2</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>Beverage Menu and Shopping List</t>
+          <t>Keg Filling</t>
         </is>
       </c>
       <c r="E43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="12" t="n"/>
-      <c r="B44" s="10" t="inlineStr">
-        <is>
-          <t>Events</t>
-        </is>
-      </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>Eve1</t>
+          <t>Bev3</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>Signup Monkey</t>
+          <t>Beverage Menu and Shopping List</t>
         </is>
       </c>
       <c r="E44" s="11" t="n"/>
@@ -1161,12 +1159,12 @@
       <c r="A45" s="12" t="n"/>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>Events</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>LNT1</t>
+          <t>Eve1</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
@@ -1178,6 +1176,21 @@
     </row>
     <row r="46">
       <c r="A46" s="12" t="n"/>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>LNT</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>LNT1</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>Signup Monkey</t>
+        </is>
+      </c>
       <c r="E46" s="11" t="n"/>
     </row>
     <row r="47">
@@ -1213,11 +1226,15 @@
       <c r="E54" s="11" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="13" t="n"/>
-      <c r="B55" s="14" t="n"/>
-      <c r="C55" s="14" t="n"/>
-      <c r="D55" s="14" t="n"/>
-      <c r="E55" s="15" t="n"/>
+      <c r="A55" s="12" t="n"/>
+      <c r="E55" s="11" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="13" t="n"/>
+      <c r="B56" s="14" t="n"/>
+      <c r="C56" s="14" t="n"/>
+      <c r="D56" s="14" t="n"/>
+      <c r="E56" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>